<commit_message>
Updated stage 2 with full data.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/HZD_Focus/tables/HZD_single_cutoff_metrics.xlsx
+++ b/results/01_pollution_assessment/HZD_Focus/tables/HZD_single_cutoff_metrics.xlsx
@@ -488,7 +488,7 @@
         <v>0.05</v>
       </c>
       <c r="C2" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -504,7 +504,7 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
@@ -519,7 +519,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -535,7 +535,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
@@ -550,7 +550,7 @@
         <v>0.09</v>
       </c>
       <c r="C4" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -566,7 +566,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
@@ -581,7 +581,7 @@
         <v>0.11</v>
       </c>
       <c r="C5" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="n">
@@ -612,7 +612,7 @@
         <v>0.13</v>
       </c>
       <c r="C6" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
@@ -643,7 +643,7 @@
         <v>0.15</v>
       </c>
       <c r="C7" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
@@ -659,7 +659,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
@@ -674,7 +674,7 @@
         <v>0.17</v>
       </c>
       <c r="C8" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -690,7 +690,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
@@ -705,7 +705,7 @@
         <v>0.19</v>
       </c>
       <c r="C9" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
@@ -721,7 +721,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
@@ -736,7 +736,7 @@
         <v>0.21</v>
       </c>
       <c r="C10" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -752,7 +752,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
@@ -767,7 +767,7 @@
         <v>0.23</v>
       </c>
       <c r="C11" t="n">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>1193.756239308613</v>
+        <v>1851.674094181419</v>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
@@ -798,28 +798,28 @@
         <v>0.25</v>
       </c>
       <c r="C12" t="n">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02269091255701996</v>
+        <v>0.01227854915103285</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005238964566966819</v>
+        <v>-0.0008910701936200027</v>
       </c>
       <c r="F12" t="n">
-        <v>1.300193684392866</v>
+        <v>0.9323389560244327</v>
       </c>
       <c r="G12" t="n">
-        <v>0.23</v>
+        <v>0.457</v>
       </c>
       <c r="H12" t="n">
-        <v>27.71632719738638</v>
+        <v>23.85272680673865</v>
       </c>
       <c r="I12" t="n">
-        <v>1221.472566506</v>
+        <v>1942.633980068581</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4862513543401121</v>
+        <v>0.3138516685097192</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
@@ -833,28 +833,28 @@
         <v>0.27</v>
       </c>
       <c r="C13" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02453033892644999</v>
+        <v>0.01251537993958646</v>
       </c>
       <c r="E13" t="n">
-        <v>0.008272511241890879</v>
+        <v>0.0003242117906924191</v>
       </c>
       <c r="F13" t="n">
-        <v>1.50883250840133</v>
+        <v>1.026593988921553</v>
       </c>
       <c r="G13" t="n">
-        <v>0.126</v>
+        <v>0.367</v>
       </c>
       <c r="H13" t="n">
-        <v>32.45789024453138</v>
+        <v>26.28955365602177</v>
       </c>
       <c r="I13" t="n">
-        <v>1323.17333004859</v>
+        <v>2100.579749310466</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5320965613857604</v>
+        <v>0.3206043128783141</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
@@ -868,28 +868,28 @@
         <v>0.29</v>
       </c>
       <c r="C14" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="D14" t="n">
-        <v>0.01620875000947223</v>
+        <v>0.01026255150361126</v>
       </c>
       <c r="E14" t="n">
-        <v>0.001073500009617923</v>
+        <v>-0.001113741007841673</v>
       </c>
       <c r="F14" t="n">
-        <v>1.070927140921246</v>
+        <v>0.9020998267475749</v>
       </c>
       <c r="G14" t="n">
-        <v>0.351</v>
+        <v>0.447</v>
       </c>
       <c r="H14" t="n">
-        <v>23.367298642189</v>
+        <v>23.1101490169068</v>
       </c>
       <c r="I14" t="n">
-        <v>1441.647173812502</v>
+        <v>2251.89116067039</v>
       </c>
       <c r="J14" t="n">
-        <v>0.354049979427106</v>
+        <v>0.2626153297375772</v>
       </c>
       <c r="K14" t="n">
         <v>1</v>
@@ -903,28 +903,28 @@
         <v>0.31</v>
       </c>
       <c r="C15" t="n">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01460547295425601</v>
+        <v>0.008516526660505305</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0005284082821739311</v>
+        <v>-0.00203116986438312</v>
       </c>
       <c r="F15" t="n">
-        <v>1.037536822802406</v>
+        <v>0.807430005253734</v>
       </c>
       <c r="G15" t="n">
-        <v>0.349</v>
+        <v>0.553</v>
       </c>
       <c r="H15" t="n">
-        <v>22.56871389911598</v>
+        <v>20.67907514038962</v>
       </c>
       <c r="I15" t="n">
-        <v>1545.223079718175</v>
+        <v>2428.111360971502</v>
       </c>
       <c r="J15" t="n">
-        <v>0.3178692098467041</v>
+        <v>0.2176744751619958</v>
       </c>
       <c r="K15" t="n">
         <v>1</v>
@@ -938,28 +938,28 @@
         <v>0.33</v>
       </c>
       <c r="C16" t="n">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01247551195550653</v>
+        <v>0.01132542177884247</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0008694135586082563</v>
+        <v>0.001438675996630834</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9348506248544681</v>
+        <v>1.145515625497258</v>
       </c>
       <c r="G16" t="n">
-        <v>0.468</v>
+        <v>0.306</v>
       </c>
       <c r="H16" t="n">
-        <v>20.33865913189402</v>
+        <v>29.09841196561993</v>
       </c>
       <c r="I16" t="n">
-        <v>1630.286532883871</v>
+        <v>2569.30051117213</v>
       </c>
       <c r="J16" t="n">
-        <v>0.271182121758587</v>
+        <v>0.2881030887685143</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
@@ -973,28 +973,28 @@
         <v>0.35</v>
       </c>
       <c r="C17" t="n">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01650073871402433</v>
+        <v>0.01272230633705602</v>
       </c>
       <c r="E17" t="n">
-        <v>0.004051380976227148</v>
+        <v>0.00340836583080173</v>
       </c>
       <c r="F17" t="n">
-        <v>1.325428914611946</v>
+        <v>1.365942409500379</v>
       </c>
       <c r="G17" t="n">
-        <v>0.205</v>
+        <v>0.2</v>
       </c>
       <c r="H17" t="n">
-        <v>28.33363958879021</v>
+        <v>34.82025428100881</v>
       </c>
       <c r="I17" t="n">
-        <v>1717.113402002351</v>
+        <v>2736.945122881416</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3541704948598777</v>
+        <v>0.3254229372056899</v>
       </c>
       <c r="K17" t="n">
         <v>1</v>
@@ -1008,28 +1008,28 @@
         <v>0.37</v>
       </c>
       <c r="C18" t="n">
-        <v>86</v>
+        <v>114</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01372764539297056</v>
+        <v>0.01227144097137004</v>
       </c>
       <c r="E18" t="n">
-        <v>0.001986307838125034</v>
+        <v>0.003452435980042967</v>
       </c>
       <c r="F18" t="n">
-        <v>1.169172194296146</v>
+        <v>1.39147681438419</v>
       </c>
       <c r="G18" t="n">
-        <v>0.267</v>
+        <v>0.174</v>
       </c>
       <c r="H18" t="n">
-        <v>24.89531983682641</v>
+        <v>35.09955648970752</v>
       </c>
       <c r="I18" t="n">
-        <v>1813.517112670642</v>
+        <v>2860.26364561397</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2928861157273693</v>
+        <v>0.3106155441567038</v>
       </c>
       <c r="K18" t="n">
         <v>1</v>
@@ -1043,28 +1043,28 @@
         <v>0.39</v>
       </c>
       <c r="C19" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01250334781456195</v>
+        <v>0.01141903990373064</v>
       </c>
       <c r="E19" t="n">
-        <v>0.001281794948818304</v>
+        <v>0.003041235157152045</v>
       </c>
       <c r="F19" t="n">
-        <v>1.114226164966108</v>
+        <v>1.36301098547255</v>
       </c>
       <c r="G19" t="n">
-        <v>0.326</v>
+        <v>0.198</v>
       </c>
       <c r="H19" t="n">
-        <v>24.23803397751677</v>
+        <v>34.02176637524554</v>
       </c>
       <c r="I19" t="n">
-        <v>1938.523532816395</v>
+        <v>2979.38939368541</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2723374604215367</v>
+        <v>0.2858971964306346</v>
       </c>
       <c r="K19" t="n">
         <v>1</v>
@@ -1078,28 +1078,28 @@
         <v>0.41</v>
       </c>
       <c r="C20" t="n">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="D20" t="n">
-        <v>0.006237432351329804</v>
+        <v>0.01281724362969731</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.00444818665564517</v>
+        <v>0.00491978157873485</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5837221360090018</v>
+        <v>1.622957292733725</v>
       </c>
       <c r="G20" t="n">
-        <v>0.82</v>
+        <v>0.116</v>
       </c>
       <c r="H20" t="n">
-        <v>12.82406472187948</v>
+        <v>40.22330178827458</v>
       </c>
       <c r="I20" t="n">
-        <v>2055.984578196735</v>
+        <v>3138.217775238193</v>
       </c>
       <c r="J20" t="n">
-        <v>0.1364262204455263</v>
+        <v>0.3192325538751951</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
@@ -1113,28 +1113,28 @@
         <v>0.43</v>
       </c>
       <c r="C21" t="n">
-        <v>100</v>
+        <v>133</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0102538231992958</v>
+        <v>0.009239009691798064</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0001543724156152226</v>
+        <v>0.001675948697078988</v>
       </c>
       <c r="F21" t="n">
-        <v>1.015285228763587</v>
+        <v>1.221596612568535</v>
       </c>
       <c r="G21" t="n">
-        <v>0.401</v>
+        <v>0.265</v>
       </c>
       <c r="H21" t="n">
-        <v>21.87719381121574</v>
+        <v>30.83240983337534</v>
       </c>
       <c r="I21" t="n">
-        <v>2133.564562798214</v>
+        <v>3337.198559359325</v>
       </c>
       <c r="J21" t="n">
-        <v>0.220981755668846</v>
+        <v>0.2335788623740556</v>
       </c>
       <c r="K21" t="n">
         <v>1</v>
@@ -1148,28 +1148,28 @@
         <v>0.45</v>
       </c>
       <c r="C22" t="n">
-        <v>233</v>
+        <v>139</v>
       </c>
       <c r="D22" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.009079397747201325</v>
       </c>
       <c r="E22" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.001846400650465485</v>
       </c>
       <c r="F22" t="n">
-        <v>8.363792289201486</v>
+        <v>1.255274629005291</v>
       </c>
       <c r="G22" t="n">
-        <v>0.001</v>
+        <v>0.239</v>
       </c>
       <c r="H22" t="n">
-        <v>213.860861192194</v>
+        <v>31.02843277539596</v>
       </c>
       <c r="I22" t="n">
-        <v>6120.49474534301</v>
+        <v>3417.454950132602</v>
       </c>
       <c r="J22" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.2248437157637388</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
@@ -1183,28 +1183,28 @@
         <v>0.47</v>
       </c>
       <c r="C23" t="n">
-        <v>233</v>
+        <v>145</v>
       </c>
       <c r="D23" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.01888882913892799</v>
       </c>
       <c r="E23" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01202791186017915</v>
       </c>
       <c r="F23" t="n">
-        <v>8.363792289201486</v>
+        <v>2.753105506378121</v>
       </c>
       <c r="G23" t="n">
-        <v>0.001</v>
+        <v>0.016</v>
       </c>
       <c r="H23" t="n">
-        <v>213.860861192194</v>
+        <v>66.31599704744841</v>
       </c>
       <c r="I23" t="n">
-        <v>6120.49474534301</v>
+        <v>3510.85800817467</v>
       </c>
       <c r="J23" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.460527757273948</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
@@ -1218,28 +1218,28 @@
         <v>0.49</v>
       </c>
       <c r="C24" t="n">
-        <v>233</v>
+        <v>151</v>
       </c>
       <c r="D24" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02235358930241991</v>
       </c>
       <c r="E24" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01579220399572467</v>
       </c>
       <c r="F24" t="n">
-        <v>8.363792289201486</v>
+        <v>3.40683990614155</v>
       </c>
       <c r="G24" t="n">
-        <v>0.001</v>
+        <v>0.006</v>
       </c>
       <c r="H24" t="n">
-        <v>213.860861192194</v>
+        <v>81.1127798851614</v>
       </c>
       <c r="I24" t="n">
-        <v>6120.49474534301</v>
+        <v>3628.624414083713</v>
       </c>
       <c r="J24" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.5407518659010763</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
@@ -1253,28 +1253,28 @@
         <v>0.51</v>
       </c>
       <c r="C25" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D25" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E25" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F25" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G25" t="n">
         <v>0.001</v>
       </c>
       <c r="H25" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I25" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J25" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -1288,28 +1288,28 @@
         <v>0.53</v>
       </c>
       <c r="C26" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D26" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E26" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F26" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G26" t="n">
         <v>0.001</v>
       </c>
       <c r="H26" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I26" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J26" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
@@ -1323,28 +1323,28 @@
         <v>0.55</v>
       </c>
       <c r="C27" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D27" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E27" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F27" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G27" t="n">
         <v>0.001</v>
       </c>
       <c r="H27" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I27" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -1358,28 +1358,28 @@
         <v>0.57</v>
       </c>
       <c r="C28" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D28" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E28" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F28" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G28" t="n">
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I28" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K28" t="n">
         <v>1</v>
@@ -1393,28 +1393,28 @@
         <v>0.59</v>
       </c>
       <c r="C29" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D29" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E29" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F29" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G29" t="n">
         <v>0.001</v>
       </c>
       <c r="H29" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I29" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J29" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
@@ -1428,28 +1428,28 @@
         <v>0.61</v>
       </c>
       <c r="C30" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D30" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E30" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F30" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G30" t="n">
         <v>0.001</v>
       </c>
       <c r="H30" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I30" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J30" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
@@ -1463,28 +1463,28 @@
         <v>0.63</v>
       </c>
       <c r="C31" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D31" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E31" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F31" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G31" t="n">
         <v>0.001</v>
       </c>
       <c r="H31" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I31" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J31" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
@@ -1498,28 +1498,28 @@
         <v>0.65</v>
       </c>
       <c r="C32" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D32" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F32" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G32" t="n">
         <v>0.001</v>
       </c>
       <c r="H32" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I32" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J32" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
@@ -1533,28 +1533,28 @@
         <v>0.67</v>
       </c>
       <c r="C33" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D33" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E33" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F33" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G33" t="n">
         <v>0.001</v>
       </c>
       <c r="H33" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I33" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J33" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
@@ -1568,28 +1568,28 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="C34" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D34" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E34" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F34" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G34" t="n">
         <v>0.001</v>
       </c>
       <c r="H34" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I34" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J34" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K34" t="n">
         <v>1</v>
@@ -1603,28 +1603,28 @@
         <v>0.71</v>
       </c>
       <c r="C35" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D35" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E35" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F35" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G35" t="n">
         <v>0.001</v>
       </c>
       <c r="H35" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I35" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J35" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K35" t="n">
         <v>1</v>
@@ -1638,28 +1638,28 @@
         <v>0.73</v>
       </c>
       <c r="C36" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D36" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E36" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F36" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G36" t="n">
         <v>0.001</v>
       </c>
       <c r="H36" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I36" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J36" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K36" t="n">
         <v>1</v>
@@ -1673,28 +1673,28 @@
         <v>0.75</v>
       </c>
       <c r="C37" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D37" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E37" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F37" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G37" t="n">
         <v>0.001</v>
       </c>
       <c r="H37" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I37" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J37" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K37" t="n">
         <v>1</v>
@@ -1708,28 +1708,28 @@
         <v>0.77</v>
       </c>
       <c r="C38" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D38" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E38" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F38" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G38" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="H38" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I38" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J38" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K38" t="n">
         <v>1</v>
@@ -1743,28 +1743,28 @@
         <v>0.79</v>
       </c>
       <c r="C39" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D39" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E39" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F39" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G39" t="n">
         <v>0.001</v>
       </c>
       <c r="H39" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I39" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J39" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K39" t="n">
         <v>1</v>
@@ -1778,28 +1778,28 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="C40" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D40" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E40" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F40" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G40" t="n">
         <v>0.001</v>
       </c>
       <c r="H40" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I40" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J40" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
@@ -1813,28 +1813,28 @@
         <v>0.83</v>
       </c>
       <c r="C41" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D41" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E41" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F41" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G41" t="n">
         <v>0.001</v>
       </c>
       <c r="H41" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I41" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J41" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K41" t="n">
         <v>1</v>
@@ -1848,28 +1848,28 @@
         <v>0.85</v>
       </c>
       <c r="C42" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D42" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E42" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F42" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G42" t="n">
         <v>0.001</v>
       </c>
       <c r="H42" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I42" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J42" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K42" t="n">
         <v>1</v>
@@ -1883,28 +1883,28 @@
         <v>0.87</v>
       </c>
       <c r="C43" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D43" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E43" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F43" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G43" t="n">
         <v>0.001</v>
       </c>
       <c r="H43" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I43" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J43" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K43" t="n">
         <v>1</v>
@@ -1918,28 +1918,28 @@
         <v>0.89</v>
       </c>
       <c r="C44" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D44" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E44" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F44" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G44" t="n">
         <v>0.001</v>
       </c>
       <c r="H44" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I44" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J44" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K44" t="n">
         <v>1</v>
@@ -1953,28 +1953,28 @@
         <v>0.91</v>
       </c>
       <c r="C45" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D45" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E45" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F45" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G45" t="n">
         <v>0.001</v>
       </c>
       <c r="H45" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I45" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J45" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K45" t="n">
         <v>1</v>
@@ -1988,28 +1988,28 @@
         <v>0.93</v>
       </c>
       <c r="C46" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D46" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E46" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F46" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G46" t="n">
         <v>0.001</v>
       </c>
       <c r="H46" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I46" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J46" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K46" t="n">
         <v>1</v>
@@ -2023,28 +2023,28 @@
         <v>0.95</v>
       </c>
       <c r="C47" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D47" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E47" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F47" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G47" t="n">
         <v>0.001</v>
       </c>
       <c r="H47" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I47" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J47" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K47" t="n">
         <v>1</v>
@@ -2058,28 +2058,28 @@
         <v>0.97</v>
       </c>
       <c r="C48" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D48" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E48" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F48" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G48" t="n">
         <v>0.001</v>
       </c>
       <c r="H48" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I48" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J48" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K48" t="n">
         <v>1</v>
@@ -2093,28 +2093,28 @@
         <v>0.99</v>
       </c>
       <c r="C49" t="n">
-        <v>233</v>
+        <v>310</v>
       </c>
       <c r="D49" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.02291017977101378</v>
       </c>
       <c r="E49" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.01973781022481569</v>
       </c>
       <c r="F49" t="n">
-        <v>8.363792289201486</v>
+        <v>7.221787826853579</v>
       </c>
       <c r="G49" t="n">
         <v>0.001</v>
       </c>
       <c r="H49" t="n">
-        <v>213.860861192194</v>
+        <v>192.652474876236</v>
       </c>
       <c r="I49" t="n">
-        <v>6120.49474534301</v>
+        <v>8409.033748394333</v>
       </c>
       <c r="J49" t="n">
-        <v>0.9218140568629059</v>
+        <v>0.6234707924797283</v>
       </c>
       <c r="K49" t="n">
         <v>1</v>

</xml_diff>